<commit_message>
organizar aeisep para projeto concluido, folha de horas e gestão de projetos
</commit_message>
<xml_diff>
--- a/DRIVE/3. Operações/3.1 Projetos/Lista entregaveis projetos.xlsx
+++ b/DRIVE/3. Operações/3.1 Projetos/Lista entregaveis projetos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\castr\MINDSET\DRIVE\3. Operações\3.1 Projetos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E17DC3-F9B4-4EB3-9F02-5F68721EFAF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C9CEDFF-3C1E-4B2C-8779-730658E698E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="55">
   <si>
     <t>Nº</t>
   </si>
@@ -196,6 +196,12 @@
   </si>
   <si>
     <t>26002 (externo)</t>
+  </si>
+  <si>
+    <t>FATURADO</t>
+  </si>
+  <si>
+    <t>Espera do cliente</t>
   </si>
 </sst>
 </file>
@@ -1342,7 +1348,7 @@
       </c>
       <c r="E6" s="12">
         <f>COUNTIF(G10:G59,"✅ Entregue")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" s="13" t="s">
         <v>13</v>
@@ -1356,10 +1362,13 @@
       </c>
       <c r="I6" s="16">
         <f>COUNTIF(G10:G59,"🔄 Em revisão")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L6" s="19" t="s">
         <v>24</v>
+      </c>
+      <c r="N6" s="31" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="9.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1440,14 +1449,14 @@
       <c r="F10" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="G10" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" s="19" t="s">
-        <v>49</v>
+      <c r="G10" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" s="35">
+        <v>46161</v>
       </c>
       <c r="I10" s="19" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="J10" s="17"/>
     </row>
@@ -1474,8 +1483,8 @@
       <c r="H11" s="35">
         <v>46147</v>
       </c>
-      <c r="I11" s="19" t="s">
-        <v>24</v>
+      <c r="I11" s="31" t="s">
+        <v>54</v>
       </c>
       <c r="J11" s="17"/>
     </row>
@@ -1503,7 +1512,7 @@
         <v>49</v>
       </c>
       <c r="I12" s="19" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="J12" s="17"/>
     </row>

</xml_diff>